<commit_message>
updadted structure and added filter
</commit_message>
<xml_diff>
--- a/docs/Gantt Chart.xlsx
+++ b/docs/Gantt Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aryan\Disseratation\intelligent-guitar-practice\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE860F06-F155-47E5-9664-463A36C191E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3799C266-300C-42A5-8805-4FD22D90FA86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{C592EF48-8C9B-48D2-B5FD-A85F508DB3A8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="85">
   <si>
     <t>Task</t>
   </si>
@@ -126,9 +126,6 @@
     <t>End</t>
   </si>
   <si>
-    <t>Complete Project Proposal &amp; Ethics Checklist</t>
-  </si>
-  <si>
     <t>Oct W1</t>
   </si>
   <si>
@@ -262,36 +259,6 @@
   </si>
   <si>
     <t>Dec W3</t>
-  </si>
-  <si>
-    <r>
-      <t>D</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Source Sans Pro"/>
-        <family val="2"/>
-      </rPr>
-      <t>**</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>L</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Source Sans Pro"/>
-        <family val="2"/>
-      </rPr>
-      <t>***</t>
-    </r>
   </si>
   <si>
     <r>
@@ -319,6 +286,60 @@
   </si>
   <si>
     <t>Feb W2</t>
+  </si>
+  <si>
+    <r>
+      <t>E</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Source Sans Pro"/>
+        <family val="2"/>
+      </rPr>
+      <t>**</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>M</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Source Sans Pro"/>
+        <family val="2"/>
+      </rPr>
+      <t>***</t>
+    </r>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <r>
+      <t>O</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Source Sans Pro"/>
+        <family val="2"/>
+      </rPr>
+      <t>*</t>
+    </r>
+  </si>
+  <si>
+    <t>Complete Project Proposal</t>
+  </si>
+  <si>
+    <t>Complete Ethics and Data Management Plan</t>
   </si>
 </sst>
 </file>
@@ -555,9 +576,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -593,6 +611,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -930,7 +949,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AL16"/>
+  <dimension ref="A1:AL17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.77734375" style="1" customWidth="1"/>
@@ -939,70 +958,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="28" t="s">
+      <c r="C1" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28" t="s">
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28" t="s">
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="P1" s="28"/>
-      <c r="Q1" s="28"/>
-      <c r="R1" s="28"/>
-      <c r="S1" s="28" t="s">
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+      <c r="S1" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="T1" s="28"/>
-      <c r="U1" s="28"/>
-      <c r="V1" s="28"/>
-      <c r="W1" s="28" t="s">
+      <c r="T1" s="27"/>
+      <c r="U1" s="27"/>
+      <c r="V1" s="27"/>
+      <c r="W1" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="X1" s="28"/>
-      <c r="Y1" s="28"/>
-      <c r="Z1" s="28"/>
-      <c r="AA1" s="28" t="s">
+      <c r="X1" s="27"/>
+      <c r="Y1" s="27"/>
+      <c r="Z1" s="27"/>
+      <c r="AA1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="AB1" s="28"/>
-      <c r="AC1" s="28"/>
-      <c r="AD1" s="28"/>
-      <c r="AE1" s="28" t="s">
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="AF1" s="28"/>
-      <c r="AG1" s="28"/>
-      <c r="AH1" s="28"/>
-      <c r="AI1" s="28" t="s">
+      <c r="AF1" s="27"/>
+      <c r="AG1" s="27"/>
+      <c r="AH1" s="27"/>
+      <c r="AI1" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="AJ1" s="28"/>
-      <c r="AK1" s="28"/>
-      <c r="AL1" s="29"/>
+      <c r="AJ1" s="27"/>
+      <c r="AK1" s="27"/>
+      <c r="AL1" s="28"/>
     </row>
     <row r="2" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A2" s="31"/>
-      <c r="B2" s="30"/>
+      <c r="A2" s="30"/>
+      <c r="B2" s="29"/>
       <c r="C2" s="2">
         <v>1</v>
       </c>
@@ -1113,14 +1132,14 @@
       </c>
     </row>
     <row r="3" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="14" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="4">
         <v>2</v>
       </c>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1157,20 +1176,20 @@
       <c r="AL3" s="3"/>
     </row>
     <row r="4" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4">
-        <v>6</v>
-      </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="25"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
+        <v>1</v>
+      </c>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
@@ -1201,22 +1220,22 @@
       <c r="AL4" s="3"/>
     </row>
     <row r="5" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="25"/>
-      <c r="L5" s="25"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1245,11 +1264,11 @@
       <c r="AL5" s="3"/>
     </row>
     <row r="6" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A6" s="15" t="s">
-        <v>75</v>
+      <c r="A6" s="14" t="s">
+        <v>14</v>
       </c>
       <c r="B6" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -1257,12 +1276,12 @@
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
+      <c r="I6" s="24"/>
+      <c r="J6" s="24"/>
+      <c r="K6" s="24"/>
       <c r="L6" s="24"/>
-      <c r="M6" s="24"/>
-      <c r="N6" s="24"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2"/>
       <c r="Q6" s="5"/>
@@ -1289,11 +1308,11 @@
       <c r="AL6" s="3"/>
     </row>
     <row r="7" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A7" s="15" t="s">
-        <v>15</v>
+      <c r="A7" s="14" t="s">
+        <v>79</v>
       </c>
       <c r="B7" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1304,14 +1323,14 @@
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
-      <c r="O7" s="25"/>
-      <c r="P7" s="25"/>
+      <c r="L7" s="23"/>
+      <c r="M7" s="23"/>
+      <c r="N7" s="23"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
       <c r="Q7" s="5"/>
       <c r="R7" s="5"/>
-      <c r="S7" s="25"/>
+      <c r="S7" s="2"/>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
@@ -1333,11 +1352,11 @@
       <c r="AL7" s="3"/>
     </row>
     <row r="8" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="14" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="4">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -1349,16 +1368,17 @@
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
       <c r="Q8" s="5"/>
       <c r="R8" s="5"/>
-      <c r="T8" s="25"/>
-      <c r="U8" s="25"/>
-      <c r="V8" s="25"/>
-      <c r="W8" s="25"/>
+      <c r="S8" s="24"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
       <c r="Z8" s="2"/>
@@ -1376,11 +1396,11 @@
       <c r="AL8" s="3"/>
     </row>
     <row r="9" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -1398,14 +1418,13 @@
       <c r="P9" s="2"/>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="25"/>
-      <c r="Y9" s="25"/>
-      <c r="Z9" s="25"/>
+      <c r="T9" s="24"/>
+      <c r="U9" s="24"/>
+      <c r="V9" s="24"/>
+      <c r="W9" s="24"/>
+      <c r="X9" s="2"/>
+      <c r="Y9" s="2"/>
+      <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
       <c r="AC9" s="2"/>
@@ -1420,11 +1439,11 @@
       <c r="AL9" s="3"/>
     </row>
     <row r="10" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="14" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -1447,11 +1466,11 @@
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-      <c r="Y10" s="2"/>
-      <c r="Z10" s="2"/>
-      <c r="AA10" s="25"/>
-      <c r="AB10" s="25"/>
+      <c r="X10" s="24"/>
+      <c r="Y10" s="24"/>
+      <c r="Z10" s="24"/>
+      <c r="AA10" s="2"/>
+      <c r="AB10" s="2"/>
       <c r="AC10" s="2"/>
       <c r="AD10" s="2"/>
       <c r="AE10" s="2"/>
@@ -1464,11 +1483,11 @@
       <c r="AL10" s="3"/>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -1494,10 +1513,10 @@
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="Z11" s="2"/>
-      <c r="AA11" s="2"/>
-      <c r="AB11" s="26"/>
-      <c r="AC11" s="26"/>
-      <c r="AD11" s="26"/>
+      <c r="AA11" s="24"/>
+      <c r="AB11" s="24"/>
+      <c r="AC11" s="2"/>
+      <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
       <c r="AF11" s="2"/>
       <c r="AG11" s="5"/>
@@ -1508,11 +1527,11 @@
       <c r="AL11" s="3"/>
     </row>
     <row r="12" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -1539,9 +1558,9 @@
       <c r="Y12" s="2"/>
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
-      <c r="AB12" s="2"/>
-      <c r="AC12" s="26"/>
-      <c r="AD12" s="26"/>
+      <c r="AB12" s="25"/>
+      <c r="AC12" s="25"/>
+      <c r="AD12" s="25"/>
       <c r="AE12" s="2"/>
       <c r="AF12" s="2"/>
       <c r="AG12" s="5"/>
@@ -1552,7 +1571,7 @@
       <c r="AL12" s="3"/>
     </row>
     <row r="13" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="4">
@@ -1584,9 +1603,10 @@
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
-      <c r="AC13" s="2"/>
-      <c r="AD13" s="26"/>
-      <c r="AE13" s="26"/>
+      <c r="AC13" s="25"/>
+      <c r="AD13" s="25"/>
+      <c r="AE13" s="2"/>
+      <c r="AF13" s="2"/>
       <c r="AG13" s="5"/>
       <c r="AH13" s="5"/>
       <c r="AI13" s="5"/>
@@ -1595,11 +1615,11 @@
       <c r="AL13" s="3"/>
     </row>
     <row r="14" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
-        <v>76</v>
+      <c r="A14" s="14" t="s">
+        <v>22</v>
       </c>
       <c r="B14" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -1627,10 +1647,9 @@
       <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
-      <c r="AC14" s="24"/>
-      <c r="AD14" s="24"/>
-      <c r="AE14" s="24"/>
-      <c r="AF14" s="24"/>
+      <c r="AC14" s="2"/>
+      <c r="AD14" s="25"/>
+      <c r="AE14" s="25"/>
       <c r="AG14" s="5"/>
       <c r="AH14" s="5"/>
       <c r="AI14" s="5"/>
@@ -1639,11 +1658,11 @@
       <c r="AL14" s="3"/>
     </row>
     <row r="15" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="s">
-        <v>23</v>
+      <c r="A15" s="14" t="s">
+        <v>80</v>
       </c>
       <c r="B15" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -1671,60 +1690,104 @@
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
-      <c r="AC15" s="2"/>
-      <c r="AD15" s="2"/>
-      <c r="AE15" s="2"/>
-      <c r="AF15" s="2"/>
-      <c r="AG15" s="24"/>
-      <c r="AH15" s="24"/>
+      <c r="AC15" s="23"/>
+      <c r="AD15" s="23"/>
+      <c r="AE15" s="23"/>
+      <c r="AF15" s="23"/>
+      <c r="AG15" s="5"/>
+      <c r="AH15" s="5"/>
       <c r="AI15" s="5"/>
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
       <c r="AL15" s="3"/>
     </row>
     <row r="16" spans="1:38" x14ac:dyDescent="0.3">
-      <c r="A16" s="16" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="6">
+      <c r="A16" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" s="4">
+        <v>2</v>
+      </c>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="5"/>
+      <c r="R16" s="5"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="2"/>
+      <c r="W16" s="2"/>
+      <c r="X16" s="2"/>
+      <c r="Y16" s="2"/>
+      <c r="Z16" s="2"/>
+      <c r="AA16" s="2"/>
+      <c r="AB16" s="2"/>
+      <c r="AC16" s="2"/>
+      <c r="AD16" s="2"/>
+      <c r="AE16" s="2"/>
+      <c r="AF16" s="2"/>
+      <c r="AG16" s="23"/>
+      <c r="AH16" s="23"/>
+      <c r="AI16" s="5"/>
+      <c r="AJ16" s="2"/>
+      <c r="AK16" s="2"/>
+      <c r="AL16" s="3"/>
+    </row>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.3">
+      <c r="A17" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="6">
         <v>1</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="8"/>
-      <c r="R16" s="8"/>
-      <c r="S16" s="7"/>
-      <c r="T16" s="7"/>
-      <c r="U16" s="7"/>
-      <c r="V16" s="7"/>
-      <c r="W16" s="7"/>
-      <c r="X16" s="7"/>
-      <c r="Y16" s="7"/>
-      <c r="Z16" s="7"/>
-      <c r="AA16" s="7"/>
-      <c r="AB16" s="7"/>
-      <c r="AC16" s="7"/>
-      <c r="AD16" s="7"/>
-      <c r="AE16" s="7"/>
-      <c r="AF16" s="7"/>
-      <c r="AG16" s="8"/>
-      <c r="AH16" s="8"/>
-      <c r="AI16" s="27"/>
-      <c r="AJ16" s="7"/>
-      <c r="AK16" s="7"/>
-      <c r="AL16" s="9"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="7"/>
+      <c r="M17" s="7"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="7"/>
+      <c r="T17" s="7"/>
+      <c r="U17" s="7"/>
+      <c r="V17" s="7"/>
+      <c r="W17" s="7"/>
+      <c r="X17" s="7"/>
+      <c r="Y17" s="7"/>
+      <c r="Z17" s="7"/>
+      <c r="AA17" s="7"/>
+      <c r="AB17" s="7"/>
+      <c r="AC17" s="7"/>
+      <c r="AD17" s="7"/>
+      <c r="AE17" s="7"/>
+      <c r="AF17" s="7"/>
+      <c r="AG17" s="8"/>
+      <c r="AH17" s="8"/>
+      <c r="AI17" s="26"/>
+      <c r="AJ17" s="7"/>
+      <c r="AK17" s="7"/>
+      <c r="AL17" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1748,7 +1811,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97EE9156-BE08-4F70-AD1D-4301D6B6195B}">
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.77734375" style="1" customWidth="1"/>
@@ -1774,10 +1837,10 @@
         <v>10</v>
       </c>
       <c r="G1" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H1" s="10" t="s">
         <v>65</v>
-      </c>
-      <c r="H1" s="10" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -1785,106 +1848,106 @@
         <v>11</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>30</v>
-      </c>
       <c r="D2" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="H2" s="18"/>
+        <v>63</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="G2" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" s="17"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>67</v>
-      </c>
-      <c r="H3" s="22"/>
+        <v>31</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="16" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="21"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>35</v>
+        <v>71</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="H4" s="19"/>
+        <v>32</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="18"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="23" t="s">
-        <v>73</v>
-      </c>
-      <c r="H5" s="20"/>
+        <v>36</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" s="19"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="G6" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="20" t="s">
         <v>70</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1892,16 +1955,16 @@
         <v>16</v>
       </c>
       <c r="B7" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>31</v>
+      <c r="E7" s="13" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1909,16 +1972,16 @@
         <v>17</v>
       </c>
       <c r="B8" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>80</v>
-      </c>
       <c r="D8" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1926,16 +1989,16 @@
         <v>18</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>47</v>
+        <v>77</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>49</v>
+        <v>44</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1943,16 +2006,16 @@
         <v>19</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C10" s="13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>48</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E10" s="14" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -1960,16 +2023,16 @@
         <v>20</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
@@ -1977,16 +2040,16 @@
         <v>21</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
@@ -1994,16 +2057,16 @@
         <v>22</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>31</v>
+        <v>54</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -2011,16 +2074,16 @@
         <v>23</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>49</v>
+        <v>55</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -2028,16 +2091,33 @@
         <v>24</v>
       </c>
       <c r="B15" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>